<commit_message>
Renommage de Paris : propager dans les Excel de temps moyens
Les fichiers Temps_moyen_par_marathon_2025 et 2026 portaient encore
« Schneider Electric Marathon de Paris ». Le rapprochement avec l'epreuve
renommee etait donc casse : ses temps moyens se seraient detaches de sa fiche
dans Vue d'ensemble et dans l'onglet Temps moyen.

Verifie apres generation : plus aucune occurrence de l'ancien nom dans le
HTML, et les series TEMPS_MARATHON, TEMPS_AVG et TIMES_DB pointent toutes sur
« ASICS Marathon de Paris ».

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Temps_moyen_par_marathon_2026.xlsx
+++ b/Temps_moyen_par_marathon_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="40" yWindow="-16310" windowWidth="29020" windowHeight="15700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finishers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Finishers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Elites" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Finishers'!$B$4:$J$4</definedName>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Schneider Electric Marathon de Paris</t>
+          <t>ASICS Marathon de Paris</t>
         </is>
       </c>
       <c r="D11" s="118" t="n">
@@ -2181,7 +2181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F59"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="23.26953125" customWidth="1" min="2" max="2"/>
@@ -2191,6 +2191,7 @@
     <col width="12.7265625" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="101" t="inlineStr">
         <is>
@@ -2198,6 +2199,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="B4" s="16" t="inlineStr">
         <is>

</xml_diff>